<commit_message>
Improve nontechnical workflow and add Claude Code support
</commit_message>
<xml_diff>
--- a/templates/ob_scale_review_template.xlsx
+++ b/templates/ob_scale_review_template.xlsx
@@ -8,12 +8,14 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variables" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questionnaire" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variables" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questionnaire" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Variables'!$A$1:$I$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Questionnaire'!$A$1:$F$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Guide'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Variables'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Questionnaire'!$A$1:$F$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,6 +34,7 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="001F4E78"/>
       <sz val="16"/>
     </font>
     <font>
@@ -55,13 +58,18 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D7DEE8"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -74,7 +82,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -442,11 +450,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="115" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -464,55 +472,43 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Use this workbook to organize variables, source scale items, translated/adapted Chinese items, respondents, waves, and references before using $ob-scale-review.</t>
+          <t>Organize variables, source scale items, Chinese translations/adaptations, respondents, waves, and references before using $ob-scale-review.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Sheet: Variables</t>
+          <t>Not required</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>One row per variable or scale block. Include item count, respondent, time wave, scale type, and source.</t>
+          <t>You can skip this template if you already have an Excel, Word, Markdown, or plain-text questionnaire draft. Ask the skill to infer the structure first.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Sheet: Questionnaire</t>
+          <t>Best workflow</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Use instruction rows for each scale, followed by item rows. Keep English source items and current Chinese items side by side.</t>
+          <t>Fill Variables first, then Questionnaire. Keep source items and current Chinese wording side by side.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>You can still use non-template files</t>
+          <t>中文说明</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>If your questionnaire is already in another format, upload it and ask Codex to infer the structure first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>中文说明</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>本模板用于整理组织行为学/管理学问卷中的变量、英文原始量表、中文翻译或改编条目、填写者、时间点和来源。</t>
+          <t>本模板用于整理变量、英文原始量表、中文翻译或改编条目、填写者、时间点、量表类型和来源。不是必须使用，但会让审阅更稳定。</t>
         </is>
       </c>
     </row>
@@ -527,204 +523,215 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>变量名称</t>
+          <t>Column / Concept</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>变量名称-中文</t>
+          <t>What to enter</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>量表条目数</t>
+          <t>Example</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>填写人（员工/领导/其他）</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Time (T1/T2/T3)</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>问卷编号</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>量表类型（成熟直译/成熟改编/自编/高度改编/混合）</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Source Reference</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
-        <is>
-          <t>备注</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="54" customHeight="1">
+          <t>Why it matters</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="58" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>AI Self-Efficacy</t>
+          <t>Scale type</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>员工AI自我效能感</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>1</v>
+          <t>Choose mature direct translation, mature adapted, self-developed, highly adapted, or mixed.</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>成熟改编</t>
+        </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>员工</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Employee_T1</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>成熟直译</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Author, A. A. (2024). Article title. Journal, volume(issue), pages.</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>sample row</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="54" customHeight="1">
+          <t>Determines whether the review focuses on translation, adaptation defensibility, or item-writing risks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Leader AI Advocacy</t>
+          <t>Respondent</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>员工感知的领导AI倡导</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>1</v>
+          <t>Who answers this scale: employee, leader, team member, customer, etc.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>员工 / 领导</t>
+        </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>员工</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Employee_T1</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>成熟改编</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Author, A. A. (2020). Article title. Journal, volume(issue), pages.</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>sample row; technology/green advocacy adapted to AI advocacy</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="54" customHeight="1">
+          <t>Prevents paired-survey respondent mismatch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Employee Performance</t>
+          <t>Wave</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>员工工作绩效</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>1</v>
+          <t>Survey wave or time point.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>T1 / T2 / T3</t>
+        </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>领导</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Leader_T3</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>成熟直译</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Author, A. A. (2009). Article title. Journal, volume(issue), pages.</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>sample row; leader-rated</t>
+          <t>Supports multi-wave design checks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Instruction row</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>A row with respondent, variable, instruction text, and source; original item is blank.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>请基于您的直属领导...</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Separates instructions from measurement items.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Item row</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>A row with English source item and current Chinese item; respondent/variable may be blank under the block.</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Top managers encourage...</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Allows item-level translation/adaptation review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Reverse-coded source item</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Keep the source marker and note if Chinese was rewritten positively.</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Reverse-coded source item; Chinese positive-worded</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Prevents reverse-scoring mistakes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>New item</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Mark any item not in the source scale.</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>new item / added global item</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Helps avoid presenting new items as mature-scale translations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Self-developed item</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Use Self-developed as source and explain construct intent in notes.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Self-developed; check social desirability</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Triggers item-writing risk checks.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I4"/>
+  <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -735,15 +742,313 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>变量名称</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>变量名称-中文</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>量表条目数</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>填写人（员工/领导/其他）</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Time (T1/T2/T3)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>问卷编号</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>量表类型（成熟直译/成熟改编/自编/高度改编/混合）</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Source Reference</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="58" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>AI Self-Efficacy</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>员工AI自我效能感</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>员工</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Employee_T1</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>成熟直译</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Author, A. A. (2024). Article title. Journal, volume(issue), pages.</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>sample row; replace with full item count</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="58" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Leader AI Advocacy</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>员工感知的领导AI倡导</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>员工</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Employee_T1</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>成熟改编</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Author, A. A. (2020). Article title. Journal, volume(issue), pages.</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>sample row; technology/green advocacy adapted to AI advocacy</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Leader AI Knowledge</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>员工感知的领导AI知识水平</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>员工</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Employee_T1</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>成熟改编</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Author, A. A. (1999). Article title. Journal, volume(issue), pages.</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>sample row; reverse-coded source item rewritten positively</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>AI Impression Management</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>员工AI印象管理</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>员工</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Employee_T2</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>自编</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Self-developed</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>sample row; check double-barreled wording, social desirability, and construct contamination</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Employee Performance</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>员工工作绩效</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>领导</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Leader_T3</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>成熟直译</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Author, A. A. (2009). Article title. Journal, volume(issue), pages.</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>sample row; leader-rated</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="74" customWidth="1" min="3" max="3"/>
+    <col width="74" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -778,7 +1083,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="54" customHeight="1">
+    <row r="2" ht="58" customHeight="1">
       <c r="A2" s="3" t="inlineStr"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -790,7 +1095,7 @@
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="3" t="inlineStr"/>
     </row>
-    <row r="3" ht="54" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>员工</t>
@@ -819,7 +1124,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="54" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="3" t="inlineStr"/>
       <c r="B4" s="3" t="inlineStr"/>
       <c r="C4" s="3" t="inlineStr">
@@ -835,7 +1140,7 @@
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="3" t="inlineStr"/>
     </row>
-    <row r="5" ht="54" customHeight="1">
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>员工</t>
@@ -864,7 +1169,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="54" customHeight="1">
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="3" t="inlineStr"/>
       <c r="B6" s="3" t="inlineStr"/>
       <c r="C6" s="3" t="inlineStr">
@@ -880,64 +1185,170 @@
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3" t="inlineStr"/>
     </row>
-    <row r="7" ht="54" customHeight="1">
-      <c r="A7" s="3" t="inlineStr"/>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>员工</t>
+        </is>
+      </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>员工感知的领导AI知识水平
+Leader AI Knowledge</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8" ht="54" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>领导</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>员工工作绩效</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>以下陈述涉及您对直属领导在AI方面知识水平的看法。请根据实际感受作答。（1=非常不符合，5=非常符合）</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Author, A. A. (1999). Article title. Journal, volume(issue), pages.</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>reverse-coded source item rewritten positively</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>I do not feel very knowledgeable about AI. (Reverse coded)</t>
+        </is>
+      </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>请回想该员工自上次问卷以来的实际工作表现，并评价以下描述的符合程度。（1=完全不符合，5=完全符合）</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Author, A. A. (2009). Article title. Journal, volume(issue), pages.</t>
-        </is>
-      </c>
+          <t>我认为我的直属领导掌握较多AI相关知识。</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>leader-rated instruction row</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="54" customHeight="1">
+          <t>Reverse-coded source item; Chinese item is positive-worded</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
       <c r="A9" s="3" t="inlineStr"/>
-      <c r="B9" s="3" t="inlineStr"/>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>This person always completes job assignments on time.</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>该员工总是能够按时完成工作任务。</t>
-        </is>
-      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr"/>
     </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>员工</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>员工AI印象管理
+AI Impression Management</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>以下陈述描述的是您在工作中向他人呈现AI使用情况的方式。请根据真实情况作答。（1=非常不同意，5=非常同意）</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Self-developed</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>self-developed instruction row</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1">
+      <c r="A11" s="3" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>我会让他人觉得我在积极使用AI，即使我实际使用AI的程度并不高。</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Self-developed item; check social desirability and wording</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>领导</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>员工工作绩效</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>请回想该员工自上次问卷以来的实际工作表现，并评价以下描述的符合程度。（1=完全不符合，5=完全符合）</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Author, A. A. (2009). Article title. Journal, volume(issue), pages.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>leader-rated instruction row</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>This person always completes job assignments on time.</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>该员工总是能够按时完成工作任务。</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F9"/>
+  <autoFilter ref="A1:F14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>